<commit_message>
Add weekly art-production load vs capacity sheet with high-load highlighting
Co-authored-by: devlee <devlee@outlook.com>
</commit_message>
<xml_diff>
--- a/上架准备工作按周排期_2026-08_2027-02.xlsx
+++ b/上架准备工作按周排期_2026-08_2027-02.xlsx
@@ -13,6 +13,7 @@
     <sheet name="批次甘特总览" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="每周工作清单" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="产能与作图拆解" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="作图负荷vs产能" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47,7 +48,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -94,6 +95,11 @@
         <fgColor rgb="00D9D2E9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -121,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -162,6 +168,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -528,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -650,49 +662,61 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="70" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>作图产能</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>单个制作: 1名设计师1款/天, 即5款/人·周, 共10人, 满投入上限50款/周(设计师另有其他需求, 有调整空间); 批量制作: 约20款/天, 满投入上限100款/周(批量线还承担在架款图片迭代, 可调整)。来图定制款按批量线处理。批次作图量按其作图周期(2-3周)均摊计算每周负荷, 详见"作图负荷vs产能"表。排期保守地要求每批作图在首个上架周前全部完成(留缓冲), 因此每月月初周作图负荷很低; 高负荷周(占用≥80%)可把当月靠后周次上架款的作图顺延到月初空档周削峰。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>春节安排</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>假设 2027/2/5-2/18 放假14天(以公司通知为准), 2/8周与2/15周不排任何工作。2月120款全部于 1/29(节前)完成作图, 分 2/1周(65款)与 2/22周(55款)两次上架。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>2027-03 批次提示</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>受春节影响, 3月批次(量待定)中妈妈装需提前: 1/18-1/29 完成选款打分定款, 节前完成SPU并启动作图, 节后 2/22周 收尾作图, 3月第1周正常上架; 常规品类节后 2/22周 立即选款(或直接定款); 婚纱可优先用来图定制款过渡。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>2027-03 批次提示</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>受春节影响, 3月批次(量待定)中妈妈装需提前: 1/18-1/29 完成选款打分定款, 节前完成SPU并启动作图, 节后 2/22周 收尾作图, 3月第1周正常上架; 常规品类节后 2/22周 立即选款(或直接定款); 婚纱可优先用来图定制款过渡。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>8月追赶(当前进度)</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>BD: 选款打分已完成→本周定款; ED: 已定款→本周SPU+作图; MBD: 作图中→8/10周起滚动上架; WD: 未启动→本周直接定款30款(来图定制另覆盖20款), 8/24周起上架, 必要时部分顺延至9月第1周。8月上架量后置明显(8/24、8/31两周合计145款), 属追赶期特殊情况。</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>图例</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>选款=浅蓝, 打分=黄色, 定款=橙色, 生成SPU=浅紫, 作图=蓝紫, 上架=绿色, 春节假期=灰色, 直接定款候选=红色。</t>
         </is>
@@ -9177,4 +9201,1126 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>周次</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>在制批次</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>单个需求(款)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>需设计师(人, 5款/人·周)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>设计师占用率(共10人)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>批量需求(款)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>批量占用(天, 20款/天)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>批量占用率(按5天)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>批量剩余产能(款, 可用于在架款迭代)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>8/3周 (8.3-8.7)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2608批、晚礼服2608批</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>54%</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>28%</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="J2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>8/10周 (8.10-8.14)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2608批、晚礼服2608批、伴娘裙2608批、婚纱2608批-选款、婚纱2608批-来图定制</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>78%</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="J3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>8/17周 (8.17-8.21)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>伴娘裙2608批、婚纱2608批-选款、婚纱2608批-来图定制、妈妈装2609批、婚纱2609批-选款</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>68%</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>43%</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>8/24周 (8.24-8.28)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>婚纱2608批-选款、妈妈装2609批、晚礼服2609批、伴娘裙2609批、婚纱2609批-选款、婚纱2609批-来图定制、花童裙2609批</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>89%</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>67%</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>单个作图高负荷: 需保证设计师投入, 排开其他需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>8/31周 (8.31-9.4)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2609批、晚礼服2609批、伴娘裙2609批、婚纱2609批-选款、婚纱2609批-来图定制、鸡尾酒裙2609批、花童裙2609批</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>70%</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>单个作图高负荷: 需保证设计师投入, 排开其他需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>9/7周 (9.7-9.11)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>鸡尾酒裙2609批</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>6%</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>7%</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="J7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>9/14周 (9.14-9.18)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2610批、婚纱2610批-选款</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>13%</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="J8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>9/21周 (9.21-9.25)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2610批、晚礼服2610批、伴娘裙2610批、婚纱2610批-选款、婚纱2610批-来图定制、小伴娘裙2610批</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>73%</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>62%</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="J9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>9/28周 (9.28-10.2)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2610批、晚礼服2610批、伴娘裙2610批、婚纱2610批-选款、婚纱2610批-来图定制、鸡尾酒裙2610批、小伴娘裙2610批</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>76%</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>65.3</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>65%</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="J10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>10/5周 (10.5-10.9)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>鸡尾酒裙2610批</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>4%</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="J11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>10/12周 (10.12-10.16)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2611批、婚纱2611批-选款、花童裙2610批</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>54%</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>23%</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>77</v>
+      </c>
+      <c r="J12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>10/19周 (10.19-10.23)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2611批、晚礼服2611批、伴娘裙2611批、婚纱2611批-选款、婚纱2611批-来图定制、花童裙2610批</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>87%</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>71.5</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>72%</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>单个作图高负荷: 需保证设计师投入, 排开其他需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>10/26周 (10.26-10.30)</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2611批、晚礼服2611批、伴娘裙2611批、婚纱2611批-选款、婚纱2611批-来图定制、舞会裙2611批</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>87%</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>71.5</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>72%</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>单个作图高负荷: 需保证设计师投入, 排开其他需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>11/2周 (11.2-11.6)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>舞会裙2611批、鸡尾酒裙2611批</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>14%</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>86</v>
+      </c>
+      <c r="J15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>11/9周 (11.9-11.13)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>鸡尾酒裙2611批、花童裙2611批</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="J16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>11/16周 (11.16-11.20)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2612批、花童裙2611批</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>14%</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>85.8</v>
+      </c>
+      <c r="J17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>11/23周 (11.23-11.27)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2612批、晚礼服2612批、伴娘裙2612批、舞会裙2612批、鸡尾酒裙2612批</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>77%</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>63%</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="J18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>11/30周 (11.30-12.4)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2612批、晚礼服2612批、伴娘裙2612批、婚纱2612批-来图定制、舞会裙2612批、鸡尾酒裙2612批</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>77%</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>68%</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="J19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>12/7周 (12.7-12.11)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>婚纱2612批-来图定制、花童裙2612批</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>6%</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="J20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>12/14周 (12.14-12.18)</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2701批、小伴娘裙2612批、花童裙2612批</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>44%</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="J21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>12/21周 (12.21-12.25)</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2701批、晚礼服2701批、伴娘裙2701批、婚纱2701批-来图定制、舞会裙2701批、小伴娘裙2612批</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>74%</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>65%</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="J22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>12/28周 (12.28-1.1)</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2701批、晚礼服2701批、伴娘裙2701批、婚纱2701批-来图定制、舞会裙2701批、鸡尾酒裙2701批</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>77%</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>68%</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="J23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>1/4周 (1.4-1.8)</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>鸡尾酒裙2701批</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="J24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>1/11周 (1.11-1.15)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2702批、花童裙2701批</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>26%</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>14%</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>86.3</v>
+      </c>
+      <c r="J25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>1/18周 (1.18-1.22)</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2702批、晚礼服2702批、伴娘裙2702批、婚纱2702批-来图定制、花童裙2701批</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>44%</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="J26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>1/25周 (1.25-1.29)</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2702批、晚礼服2702批、伴娘裙2702批、婚纱2702批-来图定制</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>33%</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="J27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>2/8周 (2.8-2.12)</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>春节假期</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="8" t="n"/>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="8" t="n"/>
+      <c r="H28" s="8" t="n"/>
+      <c r="I28" s="8" t="n"/>
+      <c r="J28" s="16" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>2/15周 (2.15-2.19)</t>
+        </is>
+      </c>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>春节假期</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="8" t="n"/>
+      <c r="G29" s="8" t="n"/>
+      <c r="H29" s="8" t="n"/>
+      <c r="I29" s="8" t="n"/>
+      <c r="J29" s="16" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update single-piece art capacity: 2 SPU/designer/day, compare vs current 30/week allocation
Co-authored-by: devlee <devlee@outlook.com>
</commit_message>
<xml_diff>
--- a/上架准备工作按周排期_2026-08_2027-02.xlsx
+++ b/上架准备工作按周排期_2026-08_2027-02.xlsx
@@ -48,7 +48,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -100,6 +100,11 @@
         <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF9999"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -127,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -170,6 +175,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -670,7 +678,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>单个制作: 1名设计师1款/天, 即5款/人·周, 共10人, 满投入上限50款/周(设计师另有其他需求, 有调整空间); 批量制作: 约20款/天, 满投入上限100款/周(批量线还承担在架款图片迭代, 可调整)。来图定制款按批量线处理。批次作图量按其作图周期(2-3周)均摊计算每周负荷, 详见"作图负荷vs产能"表。排期保守地要求每批作图在首个上架周前全部完成(留缓冲), 因此每月月初周作图负荷很低; 高负荷周(占用≥80%)可把当月靠后周次上架款的作图顺延到月初空档周削峰。</t>
+          <t>单个制作: 1名设计师2款/天, 即10款/人·周, 共10人, 理论上限100款/周; 但目前实际分配给新款的量约30款/周(设计师另有其他需求, 有调整空间)。批量制作: 约20款/天, 满投入上限100款/周(批量线还承担在架款图片迭代, 可调整)。来图定制款按批量线处理。批次作图量按其作图周期(2-3周)均摊计算每周负荷, 详见"作图负荷vs产能"表: 超过当前投放30款/周的周需提前与设计团队协调加量。排期保守地要求每批作图在首个上架周前全部完成(留缓冲), 因此每月月初周作图负荷很低; 高负荷周可把当月靠后周次上架款的作图顺延到月初空档周削峰。</t>
         </is>
       </c>
     </row>
@@ -9209,7 +9217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -9217,11 +9225,12 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9242,35 +9251,40 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>需设计师(人, 5款/人·周)</t>
+          <t>需设计师(人, 10款/人·周)</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>设计师占用率(共10人)</t>
+          <t>占理论产能(100款/周)</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
+          <t>对比当前投放(30款/周)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
           <t>批量需求(款)</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>批量占用(天, 20款/天)</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>批量占用率(按5天)</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>批量剩余产能(款, 可用于在架款迭代)</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>提示</t>
         </is>
@@ -9291,28 +9305,33 @@
         <v>27</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>5.4</v>
+        <v>2.7</v>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>54%</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="n">
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="H2" s="5" t="n">
         <v>1.4</v>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>28%</t>
         </is>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="J2" s="5" t="n">
         <v>72</v>
       </c>
-      <c r="J2" s="3" t="inlineStr"/>
+      <c r="K2" s="3" t="inlineStr"/>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -9329,28 +9348,37 @@
         <v>39</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>7.8</v>
+        <v>3.9</v>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>78%</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="n">
+          <t>39%</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>130%</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n">
         <v>56</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="H3" s="5" t="n">
         <v>2.8</v>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>56%</t>
         </is>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="J3" s="5" t="n">
         <v>44</v>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -9367,28 +9395,37 @@
         <v>34</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>6.8</v>
+        <v>3.4</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>68%</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="n">
+          <t>34%</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>113%</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n">
         <v>42.7</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="H4" s="5" t="n">
         <v>2.1</v>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>43%</t>
         </is>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="J4" s="5" t="n">
         <v>57.3</v>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>超当前投放量: 该周新款单个作图需提量至约35款</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -9405,30 +9442,35 @@
         <v>44.5</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="E5" s="15" t="inlineStr">
-        <is>
-          <t>89%</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>44%</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>148%</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n">
         <v>67.2</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="H5" s="5" t="n">
         <v>3.4</v>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>67%</t>
         </is>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="J5" s="5" t="n">
         <v>32.8</v>
       </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>单个作图高负荷: 需保证设计师投入, 排开其他需求</t>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>超当前投放量: 该周新款单个作图需提量至约45款</t>
         </is>
       </c>
     </row>
@@ -9447,30 +9489,35 @@
         <v>41.5</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="E6" s="15" t="inlineStr">
-        <is>
-          <t>83%</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>42%</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>138%</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n">
         <v>70.2</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="H6" s="5" t="n">
         <v>3.5</v>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>70%</t>
         </is>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>29.8</v>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>单个作图高负荷: 需保证设计师投入, 排开其他需求</t>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>超当前投放量: 该周新款单个作图需提量至约45款</t>
         </is>
       </c>
     </row>
@@ -9489,28 +9536,33 @@
         <v>3</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>6%</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n">
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="H7" s="5" t="n">
         <v>0.3</v>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>7%</t>
         </is>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="J7" s="5" t="n">
         <v>93</v>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -9527,28 +9579,33 @@
         <v>20</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="n">
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>67%</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n">
         <v>13.3</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="H8" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>13%</t>
         </is>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="J8" s="5" t="n">
         <v>86.7</v>
       </c>
-      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -9565,28 +9622,37 @@
         <v>36.5</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>7.3</v>
+        <v>3.6</v>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>73%</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n">
+          <t>36%</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>122%</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n">
         <v>61.8</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="H9" s="5" t="n">
         <v>3.1</v>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="I9" s="7" t="inlineStr">
         <is>
           <t>62%</t>
         </is>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="J9" s="5" t="n">
         <v>38.2</v>
       </c>
-      <c r="J9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -9603,28 +9669,37 @@
         <v>38</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>7.6</v>
+        <v>3.8</v>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>76%</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="n">
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>127%</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n">
         <v>65.3</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="H10" s="5" t="n">
         <v>3.3</v>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>65%</t>
         </is>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="J10" s="5" t="n">
         <v>34.7</v>
       </c>
-      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -9641,28 +9716,33 @@
         <v>1.5</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="n">
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="n">
         <v>3.5</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="H11" s="5" t="n">
         <v>0.2</v>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>4%</t>
         </is>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="J11" s="5" t="n">
         <v>96.5</v>
       </c>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -9679,28 +9759,33 @@
         <v>27</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>5.4</v>
+        <v>2.7</v>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>54%</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="n">
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="H12" s="5" t="n">
         <v>1.2</v>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>23%</t>
         </is>
       </c>
-      <c r="I12" s="5" t="n">
+      <c r="J12" s="5" t="n">
         <v>77</v>
       </c>
-      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -9717,30 +9802,35 @@
         <v>43.5</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="E13" s="15" t="inlineStr">
-        <is>
-          <t>87%</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>44%</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>145%</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="n">
         <v>71.5</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="H13" s="5" t="n">
         <v>3.6</v>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>72%</t>
         </is>
       </c>
-      <c r="I13" s="5" t="n">
+      <c r="J13" s="5" t="n">
         <v>28.5</v>
       </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>单个作图高负荷: 需保证设计师投入, 排开其他需求</t>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>超当前投放量: 该周新款单个作图需提量至约45款</t>
         </is>
       </c>
     </row>
@@ -9759,30 +9849,35 @@
         <v>43.5</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="E14" s="15" t="inlineStr">
-        <is>
-          <t>87%</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>44%</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>145%</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n">
         <v>71.5</v>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="H14" s="5" t="n">
         <v>3.6</v>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="I14" s="7" t="inlineStr">
         <is>
           <t>72%</t>
         </is>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="J14" s="5" t="n">
         <v>28.5</v>
       </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>单个作图高负荷: 需保证设计师投入, 排开其他需求</t>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>超当前投放量: 该周新款单个作图需提量至约45款</t>
         </is>
       </c>
     </row>
@@ -9801,28 +9896,33 @@
         <v>6</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>12%</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="n">
+          <t>6%</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="H15" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>14%</t>
         </is>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="J15" s="5" t="n">
         <v>86</v>
       </c>
-      <c r="J15" s="3" t="inlineStr"/>
+      <c r="K15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -9839,28 +9939,33 @@
         <v>4.5</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>9%</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="n">
+          <t>4%</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n">
         <v>10.5</v>
       </c>
-      <c r="G16" s="5" t="n">
+      <c r="H16" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="I16" s="7" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="J16" s="5" t="n">
         <v>89.5</v>
       </c>
-      <c r="J16" s="3" t="inlineStr"/>
+      <c r="K16" s="3" t="inlineStr"/>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -9877,28 +9982,33 @@
         <v>17.5</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>3.5</v>
+        <v>1.8</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>35%</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="n">
+          <t>18%</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>58%</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n">
         <v>14.2</v>
       </c>
-      <c r="G17" s="5" t="n">
+      <c r="H17" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="I17" s="7" t="inlineStr">
         <is>
           <t>14%</t>
         </is>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="J17" s="5" t="n">
         <v>85.8</v>
       </c>
-      <c r="J17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="inlineStr"/>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -9915,28 +10025,37 @@
         <v>38.5</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>7.7</v>
+        <v>3.9</v>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>77%</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="n">
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>128%</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="n">
         <v>63.2</v>
       </c>
-      <c r="G18" s="5" t="n">
+      <c r="H18" s="5" t="n">
         <v>3.2</v>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="I18" s="7" t="inlineStr">
         <is>
           <t>63%</t>
         </is>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="J18" s="5" t="n">
         <v>36.8</v>
       </c>
-      <c r="J18" s="3" t="inlineStr"/>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -9953,28 +10072,37 @@
         <v>38.5</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>7.7</v>
+        <v>3.9</v>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>77%</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="n">
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>128%</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="n">
         <v>68.2</v>
       </c>
-      <c r="G19" s="5" t="n">
+      <c r="H19" s="5" t="n">
         <v>3.4</v>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>68%</t>
         </is>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="J19" s="5" t="n">
         <v>31.8</v>
       </c>
-      <c r="J19" s="3" t="inlineStr"/>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -9991,28 +10119,33 @@
         <v>3</v>
       </c>
       <c r="D20" s="5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="H20" s="5" t="n">
         <v>0.6</v>
       </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>6%</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="I20" s="7" t="inlineStr">
         <is>
           <t>12%</t>
         </is>
       </c>
-      <c r="I20" s="5" t="n">
+      <c r="J20" s="5" t="n">
         <v>88</v>
       </c>
-      <c r="J20" s="3" t="inlineStr"/>
+      <c r="K20" s="3" t="inlineStr"/>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -10029,28 +10162,33 @@
         <v>22</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>44%</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="n">
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>73%</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="n">
         <v>24.7</v>
       </c>
-      <c r="G21" s="5" t="n">
+      <c r="H21" s="5" t="n">
         <v>1.2</v>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="I21" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="I21" s="5" t="n">
+      <c r="J21" s="5" t="n">
         <v>75.3</v>
       </c>
-      <c r="J21" s="3" t="inlineStr"/>
+      <c r="K21" s="3" t="inlineStr"/>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -10067,28 +10205,37 @@
         <v>37</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>7.4</v>
+        <v>3.7</v>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>74%</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="n">
+          <t>37%</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>123%</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="n">
         <v>64.7</v>
       </c>
-      <c r="G22" s="5" t="n">
+      <c r="H22" s="5" t="n">
         <v>3.2</v>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="I22" s="7" t="inlineStr">
         <is>
           <t>65%</t>
         </is>
       </c>
-      <c r="I22" s="5" t="n">
+      <c r="J22" s="5" t="n">
         <v>35.3</v>
       </c>
-      <c r="J22" s="3" t="inlineStr"/>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -10105,28 +10252,37 @@
         <v>38.5</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>7.7</v>
+        <v>3.9</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>77%</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="n">
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>128%</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="n">
         <v>68.2</v>
       </c>
-      <c r="G23" s="5" t="n">
+      <c r="H23" s="5" t="n">
         <v>3.4</v>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="I23" s="7" t="inlineStr">
         <is>
           <t>68%</t>
         </is>
       </c>
-      <c r="I23" s="5" t="n">
+      <c r="J23" s="5" t="n">
         <v>31.8</v>
       </c>
-      <c r="J23" s="3" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -10143,28 +10299,33 @@
         <v>4.5</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>9%</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="n">
+          <t>4%</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="n">
         <v>10.5</v>
       </c>
-      <c r="G24" s="5" t="n">
+      <c r="H24" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="H24" s="7" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="I24" s="5" t="n">
+      <c r="J24" s="5" t="n">
         <v>89.5</v>
       </c>
-      <c r="J24" s="3" t="inlineStr"/>
+      <c r="K24" s="3" t="inlineStr"/>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -10181,28 +10342,33 @@
         <v>13</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>26%</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="n">
+          <t>13%</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>43%</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="n">
         <v>13.7</v>
       </c>
-      <c r="G25" s="5" t="n">
+      <c r="H25" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>14%</t>
         </is>
       </c>
-      <c r="I25" s="5" t="n">
+      <c r="J25" s="5" t="n">
         <v>86.3</v>
       </c>
-      <c r="J25" s="3" t="inlineStr"/>
+      <c r="K25" s="3" t="inlineStr"/>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -10219,28 +10385,33 @@
         <v>22</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>44%</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="n">
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>73%</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="n">
         <v>39.7</v>
       </c>
-      <c r="G26" s="5" t="n">
+      <c r="H26" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H26" s="7" t="inlineStr">
+      <c r="I26" s="7" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
       </c>
-      <c r="I26" s="5" t="n">
+      <c r="J26" s="5" t="n">
         <v>60.3</v>
       </c>
-      <c r="J26" s="3" t="inlineStr"/>
+      <c r="K26" s="3" t="inlineStr"/>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -10257,36 +10428,41 @@
         <v>19</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>3.8</v>
+        <v>1.9</v>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>38%</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="n">
+          <t>19%</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>63%</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="n">
         <v>32.7</v>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="H27" s="5" t="n">
         <v>1.6</v>
       </c>
-      <c r="H27" s="7" t="inlineStr">
+      <c r="I27" s="7" t="inlineStr">
         <is>
           <t>33%</t>
         </is>
       </c>
-      <c r="I27" s="5" t="n">
+      <c r="J27" s="5" t="n">
         <v>67.3</v>
       </c>
-      <c r="J27" s="3" t="inlineStr"/>
+      <c r="K27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>2/8周 (2.8-2.12)</t>
         </is>
       </c>
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>春节假期</t>
         </is>
@@ -10298,15 +10474,16 @@
       <c r="G28" s="8" t="n"/>
       <c r="H28" s="8" t="n"/>
       <c r="I28" s="8" t="n"/>
-      <c r="J28" s="16" t="n"/>
+      <c r="J28" s="17" t="n"/>
+      <c r="K28" s="8" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>2/15周 (2.15-2.19)</t>
         </is>
       </c>
-      <c r="B29" s="16" t="inlineStr">
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>春节假期</t>
         </is>
@@ -10318,7 +10495,8 @@
       <c r="G29" s="8" t="n"/>
       <c r="H29" s="8" t="n"/>
       <c r="I29" s="8" t="n"/>
-      <c r="J29" s="16" t="n"/>
+      <c r="J29" s="17" t="n"/>
+      <c r="K29" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add smoothed weekly single-art allocation plan (EDF-leveled, flat 25/week)
Co-authored-by: devlee <devlee@outlook.com>
</commit_message>
<xml_diff>
--- a/上架准备工作按周排期_2026-08_2027-02.xlsx
+++ b/上架准备工作按周排期_2026-08_2027-02.xlsx
@@ -14,6 +14,7 @@
     <sheet name="每周工作清单" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="产能与作图拆解" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="作图负荷vs产能" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="单个作图投放计划" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -548,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -682,49 +683,61 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="56" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>单个作图投放计划</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>"作图负荷vs产能"表是按保守窗口(每批图在首个上架周前完成)计算的需求基线, 呈月中下旬高、月初低的锯齿; "单个作图投放计划"表将其平滑: 在"每款的图须在其上架周前一周的周五完成、SPU生成后才进作图队列、春节两周不排工"的约束下, 按最早截止优先排产, 得到恒定25款/周的最小可行投放量(2/1周13款收尾)。25是数学下限、无缓冲, 建议实际投放维持当前30款/周: 按25的计划表执行, 每周富余约5款用于吸收延误或在架款优化; 2月起的空档周可提前投放3月批次。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>春节安排</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>假设 2027/2/5-2/18 放假14天(以公司通知为准), 2/8周与2/15周不排任何工作。2月120款全部于 1/29(节前)完成作图, 分 2/1周(65款)与 2/22周(55款)两次上架。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>2027-03 批次提示</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>受春节影响, 3月批次(量待定)中妈妈装需提前: 1/18-1/29 完成选款打分定款, 节前完成SPU并启动作图, 节后 2/22周 收尾作图, 3月第1周正常上架; 常规品类节后 2/22周 立即选款(或直接定款); 婚纱可优先用来图定制款过渡。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>2027-03 批次提示</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>受春节影响, 3月批次(量待定)中妈妈装需提前: 1/18-1/29 完成选款打分定款, 节前完成SPU并启动作图, 节后 2/22周 收尾作图, 3月第1周正常上架; 常规品类节后 2/22周 立即选款(或直接定款); 婚纱可优先用来图定制款过渡。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>8月追赶(当前进度)</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>BD: 选款打分已完成→本周定款; ED: 已定款→本周SPU+作图; MBD: 作图中→8/10周起滚动上架; WD: 未启动→本周直接定款30款(来图定制另覆盖20款), 8/24周起上架, 必要时部分顺延至9月第1周。8月上架量后置明显(8/24、8/31两周合计145款), 属追赶期特殊情况。</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>图例</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>选款=浅蓝, 打分=黄色, 定款=橙色, 生成SPU=浅紫, 作图=蓝紫, 上架=绿色, 春节假期=灰色, 直接定款候选=红色。</t>
         </is>
@@ -10501,4 +10514,844 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="64" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>周次</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>建议投放量(款)</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>批次明细</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>对比当前投放(30款/周)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>占理论产能(100款/周)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>8/3周 (8.3-8.7)</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2608批 24、晚礼服2608批 1</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>8/10周 (8.10-8.14)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>晚礼服2608批 8、妈妈装2608批 11、伴娘裙2608批 6</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>8/17周 (8.17-8.21)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2608批 7、晚礼服2608批 3、伴娘裙2608批 6、婚纱2608批 9</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>8/24周 (8.24-8.28)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>婚纱2608批 9、妈妈装2609批 12、婚纱2609批 4</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>8/31周 (8.31-9.4)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>婚纱2609批 2.5、晚礼服2609批 3、伴娘裙2609批 3、花童裙2609批 4.5、妈妈装2609批 12</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>9/7周 (9.7-9.11)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>婚纱2609批 3.1、晚礼服2609批 3、伴娘裙2609批 3、鸡尾酒裙2609批 6、妈妈装2609批 9.9</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>9/14周 (9.14-9.18)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2609批 10.3、婚纱2609批 4.2、晚礼服2609批 3、伴娘裙2609批 3、花童裙2609批 4.5</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>9/21周 (9.21-9.25)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2609批 3.8、婚纱2609批 4.2、晚礼服2609批 3、伴娘裙2609批 3、妈妈装2610批 11</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>9/28周 (9.28-10.2)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2610批 11.5、婚纱2610批 3、晚礼服2610批 3、伴娘裙2610批 3、小伴娘裙2610批 4.5</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>10/5周 (10.5-10.9)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2610批 13、婚纱2610批 3、晚礼服2610批 3、伴娘裙2610批 3、鸡尾酒裙2610批 3</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>10/12周 (10.12-10.16)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2610批 11.5、婚纱2610批 3、晚礼服2610批 3、伴娘裙2610批 3、小伴娘裙2610批 4.5</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>10/19周 (10.19-10.23)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2610批 1、婚纱2610批 3、晚礼服2610批 3、伴娘裙2610批 3、花童裙2610批 6、妈妈装2611批 9</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>10/26周 (10.26-10.30)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2611批 15、婚纱2611批 3.4、晚礼服2611批 3.6、伴娘裙2611批 3</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>11/2周 (11.2-11.6)</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>婚纱2611批 1.4、晚礼服2611批 3.6、伴娘裙2611批 3、舞会裙2611批 6、妈妈装2611批 11</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>11/9周 (11.9-11.13)</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2611批 10、婚纱2611批 2.4、晚礼服2611批 3.6、伴娘裙2611批 3、鸡尾酒裙2611批 6</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>11/16周 (11.16-11.20)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2611批 13、婚纱2611批 2.4、晚礼服2611批 3.6、伴娘裙2611批 3、花童裙2611批 3</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>11/23周 (11.23-11.27)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2611批 2、婚纱2611批 2.4、晚礼服2611批 3.6、伴娘裙2611批 3、妈妈装2612批 12、舞会裙2612批 2</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>11/30周 (11.30-12.4)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>舞会裙2612批 1、晚礼服2612批 3.9、伴娘裙2612批 3、鸡尾酒裙2612批 6、妈妈装2612批 11.1</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>12/7周 (12.7-12.11)</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2612批 12.9、舞会裙2612批 5.2、晚礼服2612批 3.9、伴娘裙2612批 3</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>12/14周 (12.14-12.18)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>舞会裙2612批 0.8、晚礼服2612批 3.6、伴娘裙2612批 3、花童裙2612批 6、妈妈装2612批 11.6</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>12/21周 (12.21-12.25)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2612批 0.4、舞会裙2612批 3、晚礼服2612批 3.6、伴娘裙2612批 3、小伴娘裙2612批 6、妈妈装2701批 9</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>12/28周 (12.28-1.1)</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2701批 15、舞会裙2701批 4、晚礼服2701批 3、伴娘裙2701批 3</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>1/4周 (1.4-1.8)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>舞会裙2701批 2.5、晚礼服2701批 3、伴娘裙2701批 3、鸡尾酒裙2701批 4.5、妈妈装2701批 12</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>1/11周 (1.11-1.15)</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>舞会裙2701批 2.5、晚礼服2701批 3、伴娘裙2701批 3、鸡尾酒裙2701批 4.5、妈妈装2701批 12</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>1/18周 (1.18-1.22)</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>舞会裙2701批 3、晚礼服2701批 3、伴娘裙2701批 3、花童裙2701批 6、妈妈装2702批 10</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>1/25周 (1.25-1.29)</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2702批 16、晚礼服2702批 4.5、伴娘裙2702批 4.5</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2/1周 (2.1-2.5)</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>妈妈装2702批 4、晚礼服2702批 4.5、伴娘裙2702批 4.5</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>43%</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>13%</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2/8周 (2.8-2.12)</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>春节假期</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="17" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2/15周 (2.15-2.19)</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>春节假期</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="17" t="n"/>
+    </row>
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2/22周 (2.22-2.26)</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>空档: 可提前投放3月批次作图</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>3/1周 (3.1-3.5)</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>空档: 可提前投放3月批次作图</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Unify art load sheet with smoothed allocation: baseline vs smoothed columns, ratios per smoothed plan
Co-authored-by: devlee <devlee@outlook.com>
</commit_message>
<xml_diff>
--- a/上架准备工作按周排期_2026-08_2027-02.xlsx
+++ b/上架准备工作按周排期_2026-08_2027-02.xlsx
@@ -49,7 +49,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -101,11 +101,6 @@
         <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF9999"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -133,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -176,9 +171,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -679,7 +671,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>单个制作: 1名设计师2款/天, 即10款/人·周, 共10人, 理论上限100款/周; 但目前实际分配给新款的量约30款/周(设计师另有其他需求, 有调整空间)。批量制作: 约20款/天, 满投入上限100款/周(批量线还承担在架款图片迭代, 可调整)。来图定制款按批量线处理。批次作图量按其作图周期(2-3周)均摊计算每周负荷, 详见"作图负荷vs产能"表: 超过当前投放30款/周的周需提前与设计团队协调加量。排期保守地要求每批作图在首个上架周前全部完成(留缓冲), 因此每月月初周作图负荷很低; 高负荷周可把当月靠后周次上架款的作图顺延到月初空档周削峰。</t>
+          <t>单个制作: 1名设计师2款/天, 即10款/人·周, 共10人, 理论上限100款/周; 但目前实际分配给新款的量约30款/周(设计师另有其他需求, 有调整空间)。批量制作: 约20款/天, 满投入上限100款/周(批量线还承担在架款图片迭代, 可调整)。来图定制款按批量线处理。"作图负荷vs产能"表同时展示两个口径: 基线需求(保守窗口: 每批图压在首个上架周前完成, 呈月中下旬高的锯齿)与平滑后投放(SPU完成即进作图队列、按截止时间排产, 恒定25款/周); 占用率按平滑后口径计算。</t>
         </is>
       </c>
     </row>
@@ -9230,20 +9222,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="44" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9259,45 +9252,50 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>单个需求(款)</t>
+          <t>单个基线需求(款, 图压上架前完成)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>需设计师(人, 10款/人·周)</t>
+          <t>单个平滑后投放(款, 见投放计划表)</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>占理论产能(100款/周)</t>
+          <t>需设计师(人, 10款/人·周, 按平滑)</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>对比当前投放(30款/周)</t>
+          <t>占理论产能(100款/周, 按平滑)</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
+          <t>对比当前投放(30款/周, 按平滑)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
           <t>批量需求(款)</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>批量占用(天, 20款/天)</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>批量占用率(按5天)</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>批量剩余产能(款, 可用于在架款迭代)</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>提示</t>
         </is>
@@ -9318,33 +9316,36 @@
         <v>27</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>27%</t>
-        </is>
-      </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>90%</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="I2" s="5" t="n">
         <v>1.4</v>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>28%</t>
         </is>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="K2" s="5" t="n">
         <v>72</v>
       </c>
-      <c r="K2" s="3" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr"/>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -9361,35 +9362,38 @@
         <v>39</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>39%</t>
-        </is>
-      </c>
-      <c r="F3" s="16" t="inlineStr">
-        <is>
-          <t>130%</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>56</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="I3" s="5" t="n">
         <v>2.8</v>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>56%</t>
         </is>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="K3" s="5" t="n">
         <v>44</v>
       </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>基线需求39款, 已通过提前开工平滑至25款</t>
         </is>
       </c>
     </row>
@@ -9408,35 +9412,38 @@
         <v>34</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>34%</t>
-        </is>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
-        <is>
-          <t>113%</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="n">
         <v>42.7</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="I4" s="5" t="n">
         <v>2.1</v>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>43%</t>
         </is>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="K4" s="5" t="n">
         <v>57.3</v>
       </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>超当前投放量: 该周新款单个作图需提量至约35款</t>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>基线需求34款, 已通过提前开工平滑至25款</t>
         </is>
       </c>
     </row>
@@ -9455,35 +9462,38 @@
         <v>44.5</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>44%</t>
-        </is>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
-        <is>
-          <t>148%</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n">
         <v>67.2</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="I5" s="5" t="n">
         <v>3.4</v>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>67%</t>
         </is>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="K5" s="5" t="n">
         <v>32.8</v>
       </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>超当前投放量: 该周新款单个作图需提量至约45款</t>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>基线需求44款, 已通过提前开工平滑至25款</t>
         </is>
       </c>
     </row>
@@ -9502,35 +9512,38 @@
         <v>41.5</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>42%</t>
-        </is>
-      </c>
-      <c r="F6" s="16" t="inlineStr">
-        <is>
-          <t>138%</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>70.2</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="n">
         <v>3.5</v>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="J6" s="7" t="inlineStr">
         <is>
           <t>70%</t>
         </is>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="K6" s="5" t="n">
         <v>29.8</v>
       </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>超当前投放量: 该周新款单个作图需提量至约45款</t>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>基线需求42款, 已通过提前开工平滑至25款</t>
         </is>
       </c>
     </row>
@@ -9549,33 +9562,36 @@
         <v>3</v>
       </c>
       <c r="D7" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="I7" s="5" t="n">
         <v>0.3</v>
       </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>7%</t>
         </is>
       </c>
-      <c r="J7" s="5" t="n">
+      <c r="K7" s="5" t="n">
         <v>93</v>
       </c>
-      <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -9592,33 +9608,36 @@
         <v>20</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>2.5</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>67%</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n">
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>13.3</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="I8" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="J8" s="7" t="inlineStr">
         <is>
           <t>13%</t>
         </is>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="K8" s="5" t="n">
         <v>86.7</v>
       </c>
-      <c r="K8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -9635,35 +9654,38 @@
         <v>36.5</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>36%</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>122%</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="n">
         <v>61.8</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="I9" s="5" t="n">
         <v>3.1</v>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="J9" s="7" t="inlineStr">
         <is>
           <t>62%</t>
         </is>
       </c>
-      <c r="J9" s="5" t="n">
+      <c r="K9" s="5" t="n">
         <v>38.2</v>
       </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>基线需求36款, 已通过提前开工平滑至25款</t>
         </is>
       </c>
     </row>
@@ -9682,35 +9704,38 @@
         <v>38</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>38%</t>
-        </is>
-      </c>
-      <c r="F10" s="16" t="inlineStr">
-        <is>
-          <t>127%</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="n">
         <v>65.3</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="I10" s="5" t="n">
         <v>3.3</v>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>65%</t>
         </is>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="K10" s="5" t="n">
         <v>34.7</v>
       </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>基线需求38款, 已通过提前开工平滑至25款</t>
         </is>
       </c>
     </row>
@@ -9729,33 +9754,36 @@
         <v>1.5</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>2.5</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>5%</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n">
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="n">
         <v>3.5</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="I11" s="5" t="n">
         <v>0.2</v>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="J11" s="7" t="inlineStr">
         <is>
           <t>4%</t>
         </is>
       </c>
-      <c r="J11" s="5" t="n">
+      <c r="K11" s="5" t="n">
         <v>96.5</v>
       </c>
-      <c r="K11" s="3" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr"/>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -9772,33 +9800,36 @@
         <v>27</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>27%</t>
-        </is>
-      </c>
-      <c r="F12" s="15" t="inlineStr">
-        <is>
-          <t>90%</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="I12" s="5" t="n">
         <v>1.2</v>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="J12" s="7" t="inlineStr">
         <is>
           <t>23%</t>
         </is>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="K12" s="5" t="n">
         <v>77</v>
       </c>
-      <c r="K12" s="3" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr"/>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -9815,35 +9846,38 @@
         <v>43.5</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>44%</t>
-        </is>
-      </c>
-      <c r="F13" s="16" t="inlineStr">
-        <is>
-          <t>145%</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="n">
         <v>71.5</v>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="I13" s="5" t="n">
         <v>3.6</v>
       </c>
-      <c r="I13" s="7" t="inlineStr">
+      <c r="J13" s="7" t="inlineStr">
         <is>
           <t>72%</t>
         </is>
       </c>
-      <c r="J13" s="5" t="n">
+      <c r="K13" s="5" t="n">
         <v>28.5</v>
       </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>超当前投放量: 该周新款单个作图需提量至约45款</t>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>基线需求44款, 已通过提前开工平滑至25款</t>
         </is>
       </c>
     </row>
@@ -9862,35 +9896,38 @@
         <v>43.5</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>44%</t>
-        </is>
-      </c>
-      <c r="F14" s="16" t="inlineStr">
-        <is>
-          <t>145%</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="n">
         <v>71.5</v>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="I14" s="5" t="n">
         <v>3.6</v>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="J14" s="7" t="inlineStr">
         <is>
           <t>72%</t>
         </is>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="K14" s="5" t="n">
         <v>28.5</v>
       </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>超当前投放量: 该周新款单个作图需提量至约45款</t>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>基线需求44款, 已通过提前开工平滑至25款</t>
         </is>
       </c>
     </row>
@@ -9909,33 +9946,36 @@
         <v>6</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>6%</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>2.5</v>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="n">
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="I15" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="J15" s="7" t="inlineStr">
         <is>
           <t>14%</t>
         </is>
       </c>
-      <c r="J15" s="5" t="n">
+      <c r="K15" s="5" t="n">
         <v>86</v>
       </c>
-      <c r="K15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -9952,33 +9992,36 @@
         <v>4.5</v>
       </c>
       <c r="D16" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="I16" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>4%</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H16" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="J16" s="7" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="J16" s="5" t="n">
+      <c r="K16" s="5" t="n">
         <v>89.5</v>
       </c>
-      <c r="K16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr"/>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -9995,33 +10038,36 @@
         <v>17.5</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>18%</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>2.5</v>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>58%</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="n">
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>14.2</v>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="I17" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="J17" s="7" t="inlineStr">
         <is>
           <t>14%</t>
         </is>
       </c>
-      <c r="J17" s="5" t="n">
+      <c r="K17" s="5" t="n">
         <v>85.8</v>
       </c>
-      <c r="K17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr"/>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -10038,35 +10084,38 @@
         <v>38.5</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>38%</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>128%</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="n">
         <v>63.2</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="I18" s="5" t="n">
         <v>3.2</v>
       </c>
-      <c r="I18" s="7" t="inlineStr">
+      <c r="J18" s="7" t="inlineStr">
         <is>
           <t>63%</t>
         </is>
       </c>
-      <c r="J18" s="5" t="n">
+      <c r="K18" s="5" t="n">
         <v>36.8</v>
       </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
-          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>基线需求38款, 已通过提前开工平滑至25款</t>
         </is>
       </c>
     </row>
@@ -10085,35 +10134,38 @@
         <v>38.5</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>38%</t>
-        </is>
-      </c>
-      <c r="F19" s="16" t="inlineStr">
-        <is>
-          <t>128%</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="n">
         <v>68.2</v>
       </c>
-      <c r="H19" s="5" t="n">
+      <c r="I19" s="5" t="n">
         <v>3.4</v>
       </c>
-      <c r="I19" s="7" t="inlineStr">
+      <c r="J19" s="7" t="inlineStr">
         <is>
           <t>68%</t>
         </is>
       </c>
-      <c r="J19" s="5" t="n">
+      <c r="K19" s="5" t="n">
         <v>31.8</v>
       </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
-          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>基线需求38款, 已通过提前开工平滑至25款</t>
         </is>
       </c>
     </row>
@@ -10132,33 +10184,36 @@
         <v>3</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>2.5</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="n">
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="H20" s="5" t="n">
+      <c r="I20" s="5" t="n">
         <v>0.6</v>
       </c>
-      <c r="I20" s="7" t="inlineStr">
+      <c r="J20" s="7" t="inlineStr">
         <is>
           <t>12%</t>
         </is>
       </c>
-      <c r="J20" s="5" t="n">
+      <c r="K20" s="5" t="n">
         <v>88</v>
       </c>
-      <c r="K20" s="3" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr"/>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -10175,33 +10230,36 @@
         <v>22</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>22%</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>2.5</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>73%</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="n">
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="n">
         <v>24.7</v>
       </c>
-      <c r="H21" s="5" t="n">
+      <c r="I21" s="5" t="n">
         <v>1.2</v>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="J21" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="J21" s="5" t="n">
+      <c r="K21" s="5" t="n">
         <v>75.3</v>
       </c>
-      <c r="K21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr"/>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -10218,35 +10276,38 @@
         <v>37</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>37%</t>
-        </is>
-      </c>
-      <c r="F22" s="16" t="inlineStr">
-        <is>
-          <t>123%</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="n">
         <v>64.7</v>
       </c>
-      <c r="H22" s="5" t="n">
+      <c r="I22" s="5" t="n">
         <v>3.2</v>
       </c>
-      <c r="I22" s="7" t="inlineStr">
+      <c r="J22" s="7" t="inlineStr">
         <is>
           <t>65%</t>
         </is>
       </c>
-      <c r="J22" s="5" t="n">
+      <c r="K22" s="5" t="n">
         <v>35.3</v>
       </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>基线需求37款, 已通过提前开工平滑至25款</t>
         </is>
       </c>
     </row>
@@ -10265,35 +10326,38 @@
         <v>38.5</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>38%</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>128%</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="n">
         <v>68.2</v>
       </c>
-      <c r="H23" s="5" t="n">
+      <c r="I23" s="5" t="n">
         <v>3.4</v>
       </c>
-      <c r="I23" s="7" t="inlineStr">
+      <c r="J23" s="7" t="inlineStr">
         <is>
           <t>68%</t>
         </is>
       </c>
-      <c r="J23" s="5" t="n">
+      <c r="K23" s="5" t="n">
         <v>31.8</v>
       </c>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t>超当前投放量: 该周新款单个作图需提量至约40款</t>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>基线需求38款, 已通过提前开工平滑至25款</t>
         </is>
       </c>
     </row>
@@ -10312,33 +10376,36 @@
         <v>4.5</v>
       </c>
       <c r="D24" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="I24" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>4%</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H24" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I24" s="7" t="inlineStr">
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="J24" s="5" t="n">
+      <c r="K24" s="5" t="n">
         <v>89.5</v>
       </c>
-      <c r="K24" s="3" t="inlineStr"/>
+      <c r="L24" s="3" t="inlineStr"/>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -10355,33 +10422,36 @@
         <v>13</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>13%</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>2.5</v>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>43%</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="n">
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="n">
         <v>13.7</v>
       </c>
-      <c r="H25" s="5" t="n">
+      <c r="I25" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="J25" s="7" t="inlineStr">
         <is>
           <t>14%</t>
         </is>
       </c>
-      <c r="J25" s="5" t="n">
+      <c r="K25" s="5" t="n">
         <v>86.3</v>
       </c>
-      <c r="K25" s="3" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr"/>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -10398,33 +10468,36 @@
         <v>22</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>22%</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>2.5</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>73%</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="n">
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G26" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="n">
         <v>39.7</v>
       </c>
-      <c r="H26" s="5" t="n">
+      <c r="I26" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="I26" s="7" t="inlineStr">
+      <c r="J26" s="7" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
       </c>
-      <c r="J26" s="5" t="n">
+      <c r="K26" s="5" t="n">
         <v>60.3</v>
       </c>
-      <c r="K26" s="3" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr"/>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -10441,62 +10514,86 @@
         <v>19</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>19%</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>2.5</v>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>63%</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="n">
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="n">
         <v>32.7</v>
       </c>
-      <c r="H27" s="5" t="n">
+      <c r="I27" s="5" t="n">
         <v>1.6</v>
       </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="J27" s="7" t="inlineStr">
         <is>
           <t>33%</t>
         </is>
       </c>
-      <c r="J27" s="5" t="n">
+      <c r="K27" s="5" t="n">
         <v>67.3</v>
       </c>
-      <c r="K27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="17" t="inlineStr">
+      <c r="L27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2/1周 (2.1-2.5)</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>13%</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>43%</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="L28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>2/8周 (2.8-2.12)</t>
         </is>
       </c>
-      <c r="B28" s="17" t="inlineStr">
-        <is>
-          <t>春节假期</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="8" t="n"/>
-      <c r="E28" s="8" t="n"/>
-      <c r="F28" s="8" t="n"/>
-      <c r="G28" s="8" t="n"/>
-      <c r="H28" s="8" t="n"/>
-      <c r="I28" s="8" t="n"/>
-      <c r="J28" s="17" t="n"/>
-      <c r="K28" s="8" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="17" t="inlineStr">
-        <is>
-          <t>2/15周 (2.15-2.19)</t>
-        </is>
-      </c>
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B29" s="16" t="inlineStr">
         <is>
           <t>春节假期</t>
         </is>
@@ -10508,8 +10605,31 @@
       <c r="G29" s="8" t="n"/>
       <c r="H29" s="8" t="n"/>
       <c r="I29" s="8" t="n"/>
-      <c r="J29" s="17" t="n"/>
+      <c r="J29" s="16" t="n"/>
       <c r="K29" s="8" t="n"/>
+      <c r="L29" s="8" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>2/15周 (2.15-2.19)</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>春节假期</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="8" t="n"/>
+      <c r="H30" s="8" t="n"/>
+      <c r="I30" s="8" t="n"/>
+      <c r="J30" s="16" t="n"/>
+      <c r="K30" s="8" t="n"/>
+      <c r="L30" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11278,10 +11398,10 @@
           <t>春节假期</t>
         </is>
       </c>
-      <c r="C29" s="17" t="n"/>
+      <c r="C29" s="16" t="n"/>
       <c r="D29" s="8" t="n"/>
       <c r="E29" s="8" t="n"/>
-      <c r="F29" s="17" t="n"/>
+      <c r="F29" s="16" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11294,10 +11414,10 @@
           <t>春节假期</t>
         </is>
       </c>
-      <c r="C30" s="17" t="n"/>
+      <c r="C30" s="16" t="n"/>
       <c r="D30" s="8" t="n"/>
       <c r="E30" s="8" t="n"/>
-      <c r="F30" s="17" t="n"/>
+      <c r="F30" s="16" t="n"/>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Fix stale rule text, console output metrics, and selection-capacity display for completed batches
Co-authored-by: devlee <devlee@outlook.com>
</commit_message>
<xml_diff>
--- a/上架准备工作按周排期_2026-08_2027-02.xlsx
+++ b/上架准备工作按周排期_2026-08_2027-02.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="56" customHeight="1">
+    <row r="13" ht="70" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>单个作图投放计划</t>
@@ -683,7 +683,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>"作图负荷vs产能"表是按保守窗口(每批图在首个上架周前完成)计算的需求基线, 呈月中下旬高、月初低的锯齿; "单个作图投放计划"表将其平滑: 在"每款的图须在其上架周前一周的周五完成、SPU生成后才进作图队列、春节两周不排工"的约束下, 按最早截止优先排产, 得到恒定25款/周的最小可行投放量(2/1周13款收尾)。25是数学下限、无缓冲, 建议实际投放维持当前30款/周: 按25的计划表执行, 每周富余约5款用于吸收延误或在架款优化; 2月起的空档周可提前投放3月批次。</t>
+          <t>"单个作图投放计划"表给出平滑后的每周排产明细: 在"每款的图须在其上架周前一周的周五完成、SPU生成后才进作图队列、春节两周不排工"的约束下, 按最早截止优先排产, 得到恒定25款/周的最小可行投放量(2/1周13款收尾)。注意: 甘特总览与每周工作清单中的"作图"窗口是最晚完成基线, 单个作图的实际开工与排量以本投放计划表为准(SPU完成即可提前开工)。25是数学下限、无缓冲, 建议实际投放维持当前30款/周: 按25的计划表执行, 每周富余约5款用于吸收延误或在架款优化; 2月起的空档周可提前投放3月批次。</t>
         </is>
       </c>
     </row>
@@ -7519,14 +7519,20 @@
       <c r="C6" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="D6" s="5" t="n">
-        <v>60</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>1.5</v>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
@@ -10605,9 +10611,9 @@
       <c r="G29" s="8" t="n"/>
       <c r="H29" s="8" t="n"/>
       <c r="I29" s="8" t="n"/>
-      <c r="J29" s="16" t="n"/>
+      <c r="J29" s="8" t="n"/>
       <c r="K29" s="8" t="n"/>
-      <c r="L29" s="8" t="n"/>
+      <c r="L29" s="16" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
@@ -10627,9 +10633,9 @@
       <c r="G30" s="8" t="n"/>
       <c r="H30" s="8" t="n"/>
       <c r="I30" s="8" t="n"/>
-      <c r="J30" s="16" t="n"/>
+      <c r="J30" s="8" t="n"/>
       <c r="K30" s="8" t="n"/>
-      <c r="L30" s="8" t="n"/>
+      <c r="L30" s="16" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>